<commit_message>
#### Stage Loop 만드는중
</commit_message>
<xml_diff>
--- a/Assets/Scripts/Core/Parser/DropTable.xlsx
+++ b/Assets/Scripts/Core/Parser/DropTable.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wnsrl\Desktop\Dev\IdleRPG\Assets\Scripts\Core\Parser\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wnsrl\Documents\Idle_RPG_2\Assets\Scripts\Core\Parser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A034DBC1-64DA-40BB-AC93-A671E77383D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE371A8B-D4C6-4282-8C9A-8B7B6DACC094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D2027016-B747-45E9-B90F-771992799D3A}"/>
+    <workbookView xWindow="5685" yWindow="1695" windowWidth="21600" windowHeight="13785" xr2:uid="{D2027016-B747-45E9-B90F-771992799D3A}"/>
   </bookViews>
   <sheets>
     <sheet name="DropTable" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -61,6 +61,18 @@
   </si>
   <si>
     <t>SKELETON_DROPTABLE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BANDIT_ARCHER_DROPTABLE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BANDIT_LEADER_DROPTABLE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BANDIT_SHIELD_DROPTABLE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -428,10 +440,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{303C323B-7C1E-4458-A270-CCF887C3C8DC}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21.125" customWidth="1"/>
+    <col min="2" max="2" width="29" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="11.625" customWidth="1"/>
   </cols>
@@ -481,6 +493,48 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5">
+        <v>8</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Revert "Reapply "몬스터 추가""
This reverts commit 616c42261da61a9744469bace77b489276c8a2cb.
</commit_message>
<xml_diff>
--- a/Assets/Scripts/Core/Parser/DropTable.xlsx
+++ b/Assets/Scripts/Core/Parser/DropTable.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\GitHub\project-k\Assets\Scripts\Core\Parser\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wnsrl\Documents\Idle_RPG_2\Assets\Scripts\Core\Parser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E68CA960-0986-445B-B0E9-73184AE0FB08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE371A8B-D4C6-4282-8C9A-8B7B6DACC094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D2027016-B747-45E9-B90F-771992799D3A}"/>
+    <workbookView xWindow="5820" yWindow="1440" windowWidth="21600" windowHeight="13785" xr2:uid="{D2027016-B747-45E9-B90F-771992799D3A}"/>
   </bookViews>
   <sheets>
     <sheet name="DropTable" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -73,18 +73,6 @@
   </si>
   <si>
     <t>BANDIT_SHIELD_DROPTABLE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>BANDIT_KING_DROPTABLE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AMORED_ORC_DROPTABLE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ORC_KING_DROPTABLE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -452,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{303C323B-7C1E-4458-A270-CCF887C3C8DC}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="29" customWidth="1"/>
@@ -547,48 +535,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7">
-        <v>10</v>
-      </c>
-      <c r="D7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8">
-        <v>9</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9">
-        <v>15</v>
-      </c>
-      <c r="D9">
-        <v>4</v>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>